<commit_message>
chore: bump version to 2.0.70 and update layout
</commit_message>
<xml_diff>
--- a/LISTA DE LINKS.xlsx
+++ b/LISTA DE LINKS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\APRENDIZADO APP\RC-MOLINA-SEGURADORA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB6B7FC8-4396-4CBD-BC51-BB8BF5663EF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2258D3F4-13A4-4D43-A756-A1FF87750945}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2490" yWindow="60" windowWidth="21600" windowHeight="11295" xr2:uid="{1AE125DA-584A-45C4-B1F9-7B1D468BADD5}"/>
+    <workbookView xWindow="3720" yWindow="2520" windowWidth="21600" windowHeight="11295" xr2:uid="{1AE125DA-584A-45C4-B1F9-7B1D468BADD5}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Implementada rotina de limpeza no fechamento da aplicacao e atualizado icone do app
</commit_message>
<xml_diff>
--- a/LISTA DE LINKS.xlsx
+++ b/LISTA DE LINKS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\APRENDIZADO APP\RC-MOLINA-SEGURADORA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83B56678-9D46-4A8F-B4B5-F7A44FCB257F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC67BDD9-69FF-4B28-AABE-3AFE0001A5A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3720" yWindow="2520" windowWidth="21600" windowHeight="11295" xr2:uid="{1AE125DA-584A-45C4-B1F9-7B1D468BADD5}"/>
+    <workbookView xWindow="4440" yWindow="1395" windowWidth="21600" windowHeight="11295" xr2:uid="{1AE125DA-584A-45C4-B1F9-7B1D468BADD5}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -198,7 +198,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -226,6 +226,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -311,7 +326,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -334,8 +349,14 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
@@ -950,37 +971,37 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="10">
         <v>77915445715</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="10" t="s">
         <v>5</v>
       </c>
       <c r="F5" s="1"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="10">
         <v>77915445715</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="10" t="s">
         <v>5</v>
       </c>
       <c r="F6" s="1"/>
@@ -1086,16 +1107,16 @@
       <c r="F13" s="1"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="A14" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="C14" s="1">
+      <c r="C14" s="10">
         <v>77915445715</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="12" t="s">
         <v>13</v>
       </c>
       <c r="E14" s="1" t="s">
@@ -1104,16 +1125,16 @@
       <c r="F14" s="1"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+      <c r="A15" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="D15" s="10" t="s">
         <v>17</v>
       </c>
       <c r="E15" s="1" t="s">
@@ -1122,16 +1143,16 @@
       <c r="F15" s="1"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+      <c r="A16" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="1">
+      <c r="C16" s="10">
         <v>77915445715</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="D16" s="10" t="s">
         <v>33</v>
       </c>
       <c r="E16" s="1" t="s">
@@ -1140,16 +1161,16 @@
       <c r="F16" s="1"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="C17" s="1">
+      <c r="C17" s="10">
         <v>77915445715</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="12" t="s">
         <v>13</v>
       </c>
       <c r="E17" s="1" t="s">
@@ -1158,16 +1179,16 @@
       <c r="F17" s="1"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="9" t="s">
+      <c r="A18" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="14">
         <v>77915445715</v>
       </c>
-      <c r="D18" s="9" t="s">
+      <c r="D18" s="14" t="s">
         <v>13</v>
       </c>
       <c r="E18" s="9" t="s">

</xml_diff>